<commit_message>
feat(F-NAR-016): TREE-DIF-043 passe agent après apply
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-DIF-043.xlsx
+++ b/stories/arbres/TREE-DIF-043.xlsx
@@ -1197,12 +1197,12 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Sous les tilleuls, le parc sent l'herbe. Une mare brille, toute plate. Des feuilles sèches font un bruit, tout sec. Papa pose le sac, près du banc. Maman tient le seau, encore vide. Deux canards avancent, l'un derrière l'autre. Le premier a le ventre tout rond. Le second a le cou tout mince. Tu les as vus, Nino ? Oui, les deux. Je veux leur donner à manger. Les deux, Nino ? Les deux. En ce moment, Nino touche le pain. La croûte est un peu rêche, encore. Ils ne se ressemblent pas. On donne aux deux. Le pain, la nappe, et le seau. Merci, tu as vu les deux. On prépare, d'abord.</t>
+          <t>Sous les tilleuls, le parc sent l'herbe. Tu sens l'herbe, Nino ? Oui, elle est chaude. Une mare brille, toute plate. Elle est calme, là. Des feuilles sèches font un bruit, tout sec. Toc toc, les feuilles. Papa pose le sac, près du banc. Le seau est encore vide. Deux canards avancent, l'un derrière l'autre. Tu les as vus, Nino ? Oui, les deux. Le premier a le ventre tout rond. Le second a le cou tout mince. Je veux leur donner à manger. Les deux, Nino ? Les deux. En ce moment, Nino touche le pain. La croûte est un peu rêche, encore. Ils ne se ressemblent pas. On donne aux deux. Le pain, la nappe, et le seau. Merci, tu as vu les deux. On prépare, d'abord.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Sous les tilleuls, le parc sent l'herbe. Une mare brille, toute plate. Des feuilles sèches font un bruit, tout sec. Papa pose le sac, près du banc. Maman tient le seau, encore vide. Deux canards avancent, l'un derrière l'autre. Le premier a le ventre tout rond. Le second a le cou tout mince. Tu les as vus, Nino ? Oui, les deux. Je veux leur donner à manger. Les deux, Nino ? Les deux. En ce moment, Nino touche le pain. La croûte est un peu rêche, encore. Ils ne se ressemblent pas. On donne aux deux. Le pain, la nappe, et le seau. Merci, tu as vu les deux. On prépare, d'abord.</t>
+          <t>Sous les tilleuls, le parc sent l'herbe. Tu sens l'herbe, Nino ? Oui, elle est chaude. Une mare brille, toute plate. Elle est calme, là. Des feuilles sèches font un bruit, tout sec. Toc toc, les feuilles. Papa pose le sac, près du banc. Le seau est encore vide. Deux canards avancent, l'un derrière l'autre. Tu les as vus, Nino ? Oui, les deux. Le premier a le ventre tout rond. Le second a le cou tout mince. Je veux leur donner à manger. Les deux, Nino ? Les deux. En ce moment, Nino touche le pain. La croûte est un peu rêche, encore. Ils ne se ressemblent pas. On donne aux deux. Le pain, la nappe, et le seau. Merci, tu as vu les deux. On prépare, d'abord.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -1338,15 +1338,19 @@
       <c r="AW2" t="inlineStr">
         <is>
           <t>narrateur|Sous les tilleuls, le parc sent l'herbe.
+papa|Tu sens l'herbe, Nino ?
+enfant-m|Oui, elle est chaude.
 narrateur|Une mare brille, toute plate.
+maman|Elle est calme, là.
 narrateur|Des feuilles sèches font un bruit, tout sec.
+enfant-m|Toc toc, les feuilles.
 narrateur|Papa pose le sac, près du banc.
-narrateur|Maman tient le seau, encore vide.
+maman|Le seau est encore vide.
 narrateur|Deux canards avancent, l'un derrière l'autre.
+papa|Tu les as vus, Nino ?
+enfant-m|Oui, les deux.
 narrateur|Le premier a le ventre tout rond.
 narrateur|Le second a le cou tout mince.
-papa|Tu les as vus, Nino ?
-enfant-m|Oui, les deux.
 enfant-m|Je veux leur donner à manger.
 papa|Les deux, Nino ?
 enfant-m|Les deux.
@@ -2314,12 +2318,12 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Le pain sent encore le four, tout chaud. Ils s'approchent de la mare, trop haute. Un morceau de pain tombe, trop loin. L'eau fait un pli, trop vif. Vous venez. Le canard rond reste au bord. Le mince part, trop léger, trop loin. L'un reste, l'autre part. Ils n'ont pas la même forme. Tu fais quoi, avec les deux ?</t>
+          <t>Le pain sent encore le four, tout chaud. Ils s'approchent de la mare, trop haute. L'eau est grande. Un morceau de pain tombe, trop loin. L'eau fait un pli, trop vif. Vous venez. Le canard rond reste au bord. Le mince part, trop léger, trop loin. L'un reste, l'autre part. Ils n'ont pas la même forme. Tu fais quoi, avec les deux ?</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Le pain sent encore le four, tout chaud. Ils s'approchent de la mare, trop haute. Un morceau de pain tombe, trop loin. L'eau fait un pli, trop vif. Vous venez. Le canard rond reste au bord. Le mince part, trop léger, trop loin. L'un reste, l'autre part. Ils n'ont pas la même forme. Tu fais quoi, avec les deux ?</t>
+          <t>Le pain sent encore le four, tout chaud. Ils s'approchent de la mare, trop haute. L'eau est grande. Un morceau de pain tombe, trop loin. L'eau fait un pli, trop vif. Vous venez. Le canard rond reste au bord. Le mince part, trop léger, trop loin. L'un reste, l'autre part. Ils n'ont pas la même forme. Tu fais quoi, avec les deux ?</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -2456,6 +2460,7 @@
         <is>
           <t>narrateur|Le pain sent encore le four, tout chaud.
 narrateur|Ils s'approchent de la mare, trop haute.
+enfant-m|L'eau est grande.
 narrateur|Un morceau de pain tombe, trop loin.
 narrateur|L'eau fait un pli, trop vif.
 enfant-m|Vous venez.
@@ -3731,12 +3736,12 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Le pain sent encore le four, tout chaud. Sur le banc, les planches ont des fentes. Des miettes tombent entre les planches. Le goûter, ici. Nino s'assoit, trop haut pour eux. Le canard rond bute, trop large. Le mince glisse entre les planches. Ce n'est pas juste. Le banc a des trous, voilà tout. Tu les gardes comment, ensemble ?</t>
+          <t>Le pain sent encore le four, tout chaud. Sur le banc, les planches ont des fentes. Le goûter, ici. Des miettes tombent entre les planches. Nino s'assoit, trop haut pour eux. Tu es trop haut, pour eux. Le canard rond bute, trop large. Le mince glisse entre les planches. Ce n'est pas juste. Le banc a des trous, voilà tout. Tu les gardes comment, ensemble ?</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Le pain sent encore le four, tout chaud. Sur le banc, les planches ont des fentes. Des miettes tombent entre les planches. Le goûter, ici. Nino s'assoit, trop haut pour eux. Le canard rond bute, trop large. Le mince glisse entre les planches. Ce n'est pas juste. Le banc a des trous, voilà tout. Tu les gardes comment, ensemble ?</t>
+          <t>Le pain sent encore le four, tout chaud. Sur le banc, les planches ont des fentes. Le goûter, ici. Des miettes tombent entre les planches. Nino s'assoit, trop haut pour eux. Tu es trop haut, pour eux. Le canard rond bute, trop large. Le mince glisse entre les planches. Ce n'est pas juste. Le banc a des trous, voilà tout. Tu les gardes comment, ensemble ?</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -3873,9 +3878,10 @@
         <is>
           <t>narrateur|Le pain sent encore le four, tout chaud.
 narrateur|Sur le banc, les planches ont des fentes.
+enfant-m|Le goûter, ici.
 narrateur|Des miettes tombent entre les planches.
-enfant-m|Le goûter, ici.
 narrateur|Nino s'assoit, trop haut pour eux.
+papa|Tu es trop haut, pour eux.
 narrateur|Le canard rond bute, trop large.
 narrateur|Le mince glisse entre les planches.
 enfant-m|Ce n'est pas juste.
@@ -4104,12 +4110,12 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>L'herbe, comme une table. Il pose le pain dans l'herbe, tout bas. Nino s'assoit, les pieds dans l'herbe. Le canard rond s'assoit, trop rond. Le mince s'allonge contre lui, trop mince. Vous avez le sol, tous les deux. Chacun a sa place. Un peu de croûte reste, tout rêche. Les miettes restent, plus calmes.</t>
+          <t>L'herbe, comme une table. Il pose le pain dans l'herbe, tout bas. Nino s'assoit, les pieds dans l'herbe. Tout doux, dans l'herbe. Le canard rond s'assoit, trop rond. Le mince s'allonge contre lui, trop mince. Vous avez le sol, tous les deux. Chacun a sa place. Un peu de croûte reste, tout rêche. Les miettes restent, plus calmes.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>L'herbe, comme une table. Il pose le pain dans l'herbe, tout bas. Nino s'assoit, les pieds dans l'herbe. Le canard rond s'assoit, trop rond. Le mince s'allonge contre lui, trop mince. Vous avez le sol, tous les deux. Chacun a sa place. Un peu de croûte reste, tout rêche. Les miettes restent, plus calmes.</t>
+          <t>L'herbe, comme une table. Il pose le pain dans l'herbe, tout bas. Nino s'assoit, les pieds dans l'herbe. Tout doux, dans l'herbe. Le canard rond s'assoit, trop rond. Le mince s'allonge contre lui, trop mince. Vous avez le sol, tous les deux. Chacun a sa place. Un peu de croûte reste, tout rêche. Les miettes restent, plus calmes.</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -4247,6 +4253,7 @@
           <t>enfant-m|L'herbe, comme une table.
 narrateur|Il pose le pain dans l'herbe, tout bas.
 narrateur|Nino s'assoit, les pieds dans l'herbe.
+papa|Tout doux, dans l'herbe.
 narrateur|Le canard rond s'assoit, trop rond.
 narrateur|Le mince s'allonge contre lui, trop mince.
 enfant-m|Vous avez le sol, tous les deux.
@@ -5147,12 +5154,12 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Le pain sent encore le four, tout chaud. Au kiosque, les marches sont trop hautes. Le pain sent encore, trop loin de l'eau. Le goûter, là-haut. Un vent passe, tout froid. Le canard rond ne monte pas. Le mince commence, puis recule. Ils ne viennent pas. Le kiosque est trop loin de l'eau. Tu les rassembles comment ?</t>
+          <t>Le pain sent encore le four, tout chaud. Au kiosque, les marches sont trop hautes. Le goûter, là-haut. Le pain sent encore, trop loin de l'eau. Un vent passe, tout froid. Trop haut, trop loin. Le canard rond ne monte pas. Le mince commence, puis recule. Ils ne viennent pas. Le kiosque est trop loin de l'eau. Tu les rassembles comment ?</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Le pain sent encore le four, tout chaud. Au kiosque, les marches sont trop hautes. Le pain sent encore, trop loin de l'eau. Le goûter, là-haut. Un vent passe, tout froid. Le canard rond ne monte pas. Le mince commence, puis recule. Ils ne viennent pas. Le kiosque est trop loin de l'eau. Tu les rassembles comment ?</t>
+          <t>Le pain sent encore le four, tout chaud. Au kiosque, les marches sont trop hautes. Le goûter, là-haut. Le pain sent encore, trop loin de l'eau. Un vent passe, tout froid. Trop haut, trop loin. Le canard rond ne monte pas. Le mince commence, puis recule. Ils ne viennent pas. Le kiosque est trop loin de l'eau. Tu les rassembles comment ?</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -5289,9 +5296,10 @@
         <is>
           <t>narrateur|Le pain sent encore le four, tout chaud.
 narrateur|Au kiosque, les marches sont trop hautes.
+enfant-m|Le goûter, là-haut.
 narrateur|Le pain sent encore, trop loin de l'eau.
-enfant-m|Le goûter, là-haut.
 narrateur|Un vent passe, tout froid.
+maman|Trop haut, trop loin.
 narrateur|Le canard rond ne monte pas.
 narrateur|Le mince commence, puis recule.
 enfant-m|Ils ne viennent pas.
@@ -7295,12 +7303,12 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Un coin de nappe frotte l'herbe. Ils s'approchent de la mare, trop haute. La nappe accroche l'herbe, puis lâche. L'eau fait un pli, trop vif. Vous venez. Le canard rond reste au bord. Le mince part, trop léger, trop loin. L'un reste, l'autre part. Ils n'ont pas la même forme. Tu fais quoi, avec les deux ?</t>
+          <t>Un coin de nappe frotte l'herbe. Ils s'approchent de la mare, trop haute. L'eau est grande. La nappe accroche l'herbe, puis lâche. L'eau fait un pli, trop vif. Vous venez. Le canard rond reste au bord. Le mince part, trop léger, trop loin. L'un reste, l'autre part. Ils n'ont pas la même forme. Tu fais quoi, avec les deux ?</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Un coin de nappe frotte l'herbe. Ils s'approchent de la mare, trop haute. La nappe accroche l'herbe, puis lâche. L'eau fait un pli, trop vif. Vous venez. Le canard rond reste au bord. Le mince part, trop léger, trop loin. L'un reste, l'autre part. Ils n'ont pas la même forme. Tu fais quoi, avec les deux ?</t>
+          <t>Un coin de nappe frotte l'herbe. Ils s'approchent de la mare, trop haute. L'eau est grande. La nappe accroche l'herbe, puis lâche. L'eau fait un pli, trop vif. Vous venez. Le canard rond reste au bord. Le mince part, trop léger, trop loin. L'un reste, l'autre part. Ils n'ont pas la même forme. Tu fais quoi, avec les deux ?</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -7437,6 +7445,7 @@
         <is>
           <t>narrateur|Un coin de nappe frotte l'herbe.
 narrateur|Ils s'approchent de la mare, trop haute.
+enfant-m|L'eau est grande.
 narrateur|La nappe accroche l'herbe, puis lâche.
 narrateur|L'eau fait un pli, trop vif.
 enfant-m|Vous venez.
@@ -8712,12 +8721,12 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Un coin de nappe frotte l'herbe. Sur le banc, les planches ont des fentes. La nappe glisse dans le vide, trop mince. Le goûter, ici. Nino s'assoit, trop haut pour eux. Le canard rond bute, trop large. Le mince glisse entre les planches. Ce n'est pas juste. Le banc a des trous, voilà tout. Tu les gardes comment, ensemble ?</t>
+          <t>Un coin de nappe frotte l'herbe. Sur le banc, les planches ont des fentes. Le goûter, ici. La nappe glisse dans le vide, trop mince. Nino s'assoit, trop haut pour eux. Tu es trop haut, pour eux. Le canard rond bute, trop large. Le mince glisse entre les planches. Ce n'est pas juste. Le banc a des trous, voilà tout. Tu les gardes comment, ensemble ?</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Un coin de nappe frotte l'herbe. Sur le banc, les planches ont des fentes. La nappe glisse dans le vide, trop mince. Le goûter, ici. Nino s'assoit, trop haut pour eux. Le canard rond bute, trop large. Le mince glisse entre les planches. Ce n'est pas juste. Le banc a des trous, voilà tout. Tu les gardes comment, ensemble ?</t>
+          <t>Un coin de nappe frotte l'herbe. Sur le banc, les planches ont des fentes. Le goûter, ici. La nappe glisse dans le vide, trop mince. Nino s'assoit, trop haut pour eux. Tu es trop haut, pour eux. Le canard rond bute, trop large. Le mince glisse entre les planches. Ce n'est pas juste. Le banc a des trous, voilà tout. Tu les gardes comment, ensemble ?</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -8854,9 +8863,10 @@
         <is>
           <t>narrateur|Un coin de nappe frotte l'herbe.
 narrateur|Sur le banc, les planches ont des fentes.
+enfant-m|Le goûter, ici.
 narrateur|La nappe glisse dans le vide, trop mince.
-enfant-m|Le goûter, ici.
 narrateur|Nino s'assoit, trop haut pour eux.
+papa|Tu es trop haut, pour eux.
 narrateur|Le canard rond bute, trop large.
 narrateur|Le mince glisse entre les planches.
 enfant-m|Ce n'est pas juste.
@@ -9085,12 +9095,12 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>L'herbe, comme une table. Il étale la nappe dans l'herbe, tout bas. Nino s'assoit, les pieds dans l'herbe. Le canard rond s'assoit, trop rond. Le mince s'allonge contre lui, trop mince. Vous avez le sol, tous les deux. Chacun a sa place. La nappe les abrite, tout doux. Les miettes restent, plus calmes.</t>
+          <t>L'herbe, comme une table. Il étale la nappe dans l'herbe, tout bas. Nino s'assoit, les pieds dans l'herbe. Tout doux, dans l'herbe. Le canard rond s'assoit, trop rond. Le mince s'allonge contre lui, trop mince. Vous avez le sol, tous les deux. Chacun a sa place. La nappe les abrite, tout doux. Les miettes restent, plus calmes.</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>L'herbe, comme une table. Il étale la nappe dans l'herbe, tout bas. Nino s'assoit, les pieds dans l'herbe. Le canard rond s'assoit, trop rond. Le mince s'allonge contre lui, trop mince. Vous avez le sol, tous les deux. Chacun a sa place. La nappe les abrite, tout doux. Les miettes restent, plus calmes.</t>
+          <t>L'herbe, comme une table. Il étale la nappe dans l'herbe, tout bas. Nino s'assoit, les pieds dans l'herbe. Tout doux, dans l'herbe. Le canard rond s'assoit, trop rond. Le mince s'allonge contre lui, trop mince. Vous avez le sol, tous les deux. Chacun a sa place. La nappe les abrite, tout doux. Les miettes restent, plus calmes.</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -9228,6 +9238,7 @@
           <t>enfant-m|L'herbe, comme une table.
 narrateur|Il étale la nappe dans l'herbe, tout bas.
 narrateur|Nino s'assoit, les pieds dans l'herbe.
+papa|Tout doux, dans l'herbe.
 narrateur|Le canard rond s'assoit, trop rond.
 narrateur|Le mince s'allonge contre lui, trop mince.
 enfant-m|Vous avez le sol, tous les deux.
@@ -10128,12 +10139,12 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Un coin de nappe frotte l'herbe. Au kiosque, les marches sont trop hautes. La nappe claque sur les marches, trop haut. Le goûter, là-haut. Un vent passe, tout froid. Le canard rond ne monte pas. Le mince commence, puis recule. Ils ne viennent pas. Le kiosque est trop loin de l'eau. Tu les rassembles comment ?</t>
+          <t>Un coin de nappe frotte l'herbe. Au kiosque, les marches sont trop hautes. Le goûter, là-haut. La nappe claque sur les marches, trop haut. Un vent passe, tout froid. Trop haut, trop loin. Le canard rond ne monte pas. Le mince commence, puis recule. Ils ne viennent pas. Le kiosque est trop loin de l'eau. Tu les rassembles comment ?</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>Un coin de nappe frotte l'herbe. Au kiosque, les marches sont trop hautes. La nappe claque sur les marches, trop haut. Le goûter, là-haut. Un vent passe, tout froid. Le canard rond ne monte pas. Le mince commence, puis recule. Ils ne viennent pas. Le kiosque est trop loin de l'eau. Tu les rassembles comment ?</t>
+          <t>Un coin de nappe frotte l'herbe. Au kiosque, les marches sont trop hautes. Le goûter, là-haut. La nappe claque sur les marches, trop haut. Un vent passe, tout froid. Trop haut, trop loin. Le canard rond ne monte pas. Le mince commence, puis recule. Ils ne viennent pas. Le kiosque est trop loin de l'eau. Tu les rassembles comment ?</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -10270,9 +10281,10 @@
         <is>
           <t>narrateur|Un coin de nappe frotte l'herbe.
 narrateur|Au kiosque, les marches sont trop hautes.
+enfant-m|Le goûter, là-haut.
 narrateur|La nappe claque sur les marches, trop haut.
-enfant-m|Le goûter, là-haut.
 narrateur|Un vent passe, tout froid.
+maman|Trop haut, trop loin.
 narrateur|Le canard rond ne monte pas.
 narrateur|Le mince commence, puis recule.
 enfant-m|Ils ne viennent pas.
@@ -12276,12 +12288,12 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Le seau tape sa jambe, à chaque pas. Ils s'approchent de la mare, trop haute. Le seau penche, une miette tombe. L'eau fait un pli, trop vif. Vous venez. Le canard rond reste au bord. Le mince part, trop léger, trop loin. L'un reste, l'autre part. Ils n'ont pas la même forme. Tu fais quoi, avec les deux ?</t>
+          <t>Le seau tape sa jambe, à chaque pas. Ils s'approchent de la mare, trop haute. L'eau est grande. Le seau penche, une miette tombe. L'eau fait un pli, trop vif. Vous venez. Le canard rond reste au bord. Le mince part, trop léger, trop loin. L'un reste, l'autre part. Ils n'ont pas la même forme. Tu fais quoi, avec les deux ?</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>Le seau tape sa jambe, à chaque pas. Ils s'approchent de la mare, trop haute. Le seau penche, une miette tombe. L'eau fait un pli, trop vif. Vous venez. Le canard rond reste au bord. Le mince part, trop léger, trop loin. L'un reste, l'autre part. Ils n'ont pas la même forme. Tu fais quoi, avec les deux ?</t>
+          <t>Le seau tape sa jambe, à chaque pas. Ils s'approchent de la mare, trop haute. L'eau est grande. Le seau penche, une miette tombe. L'eau fait un pli, trop vif. Vous venez. Le canard rond reste au bord. Le mince part, trop léger, trop loin. L'un reste, l'autre part. Ils n'ont pas la même forme. Tu fais quoi, avec les deux ?</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -12418,6 +12430,7 @@
         <is>
           <t>narrateur|Le seau tape sa jambe, à chaque pas.
 narrateur|Ils s'approchent de la mare, trop haute.
+enfant-m|L'eau est grande.
 narrateur|Le seau penche, une miette tombe.
 narrateur|L'eau fait un pli, trop vif.
 enfant-m|Vous venez.
@@ -13693,12 +13706,12 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>Le seau tape sa jambe, à chaque pas. Sur le banc, les planches ont des fentes. Le seau cogne le bois, un toc. Le goûter, ici. Nino s'assoit, trop haut pour eux. Le canard rond bute, trop large. Le mince glisse entre les planches. Ce n'est pas juste. Le banc a des trous, voilà tout. Tu les gardes comment, ensemble ?</t>
+          <t>Le seau tape sa jambe, à chaque pas. Sur le banc, les planches ont des fentes. Le goûter, ici. Le seau cogne le bois, un toc. Nino s'assoit, trop haut pour eux. Tu es trop haut, pour eux. Le canard rond bute, trop large. Le mince glisse entre les planches. Ce n'est pas juste. Le banc a des trous, voilà tout. Tu les gardes comment, ensemble ?</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>Le seau tape sa jambe, à chaque pas. Sur le banc, les planches ont des fentes. Le seau cogne le bois, un toc. Le goûter, ici. Nino s'assoit, trop haut pour eux. Le canard rond bute, trop large. Le mince glisse entre les planches. Ce n'est pas juste. Le banc a des trous, voilà tout. Tu les gardes comment, ensemble ?</t>
+          <t>Le seau tape sa jambe, à chaque pas. Sur le banc, les planches ont des fentes. Le goûter, ici. Le seau cogne le bois, un toc. Nino s'assoit, trop haut pour eux. Tu es trop haut, pour eux. Le canard rond bute, trop large. Le mince glisse entre les planches. Ce n'est pas juste. Le banc a des trous, voilà tout. Tu les gardes comment, ensemble ?</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -13835,9 +13848,10 @@
         <is>
           <t>narrateur|Le seau tape sa jambe, à chaque pas.
 narrateur|Sur le banc, les planches ont des fentes.
+enfant-m|Le goûter, ici.
 narrateur|Le seau cogne le bois, un toc.
-enfant-m|Le goûter, ici.
 narrateur|Nino s'assoit, trop haut pour eux.
+papa|Tu es trop haut, pour eux.
 narrateur|Le canard rond bute, trop large.
 narrateur|Le mince glisse entre les planches.
 enfant-m|Ce n'est pas juste.
@@ -14066,12 +14080,12 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>L'herbe, comme une table. Il pose le seau dans l'herbe, tout bas. Nino s'assoit, les pieds dans l'herbe. Le canard rond s'assoit, trop rond. Le mince s'allonge contre lui, trop mince. Vous avez le sol, tous les deux. Chacun a sa place. Un peu d'eau tremble au bord du seau. Les miettes restent, plus calmes.</t>
+          <t>L'herbe, comme une table. Il pose le seau dans l'herbe, tout bas. Nino s'assoit, les pieds dans l'herbe. Tout doux, dans l'herbe. Le canard rond s'assoit, trop rond. Le mince s'allonge contre lui, trop mince. Vous avez le sol, tous les deux. Chacun a sa place. Un peu d'eau tremble au bord du seau. Les miettes restent, plus calmes.</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>L'herbe, comme une table. Il pose le seau dans l'herbe, tout bas. Nino s'assoit, les pieds dans l'herbe. Le canard rond s'assoit, trop rond. Le mince s'allonge contre lui, trop mince. Vous avez le sol, tous les deux. Chacun a sa place. Un peu d'eau tremble au bord du seau. Les miettes restent, plus calmes.</t>
+          <t>L'herbe, comme une table. Il pose le seau dans l'herbe, tout bas. Nino s'assoit, les pieds dans l'herbe. Tout doux, dans l'herbe. Le canard rond s'assoit, trop rond. Le mince s'allonge contre lui, trop mince. Vous avez le sol, tous les deux. Chacun a sa place. Un peu d'eau tremble au bord du seau. Les miettes restent, plus calmes.</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
@@ -14209,6 +14223,7 @@
           <t>enfant-m|L'herbe, comme une table.
 narrateur|Il pose le seau dans l'herbe, tout bas.
 narrateur|Nino s'assoit, les pieds dans l'herbe.
+papa|Tout doux, dans l'herbe.
 narrateur|Le canard rond s'assoit, trop rond.
 narrateur|Le mince s'allonge contre lui, trop mince.
 enfant-m|Vous avez le sol, tous les deux.
@@ -15109,12 +15124,12 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>Le seau tape sa jambe, à chaque pas. Au kiosque, les marches sont trop hautes. Le seau tape une marche, trop haute. Le goûter, là-haut. Un vent passe, tout froid. Le canard rond ne monte pas. Le mince commence, puis recule. Ils ne viennent pas. Le kiosque est trop loin de l'eau. Tu les rassembles comment ?</t>
+          <t>Le seau tape sa jambe, à chaque pas. Au kiosque, les marches sont trop hautes. Le goûter, là-haut. Le seau tape une marche, trop haute. Un vent passe, tout froid. Trop haut, trop loin. Le canard rond ne monte pas. Le mince commence, puis recule. Ils ne viennent pas. Le kiosque est trop loin de l'eau. Tu les rassembles comment ?</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>Le seau tape sa jambe, à chaque pas. Au kiosque, les marches sont trop hautes. Le seau tape une marche, trop haute. Le goûter, là-haut. Un vent passe, tout froid. Le canard rond ne monte pas. Le mince commence, puis recule. Ils ne viennent pas. Le kiosque est trop loin de l'eau. Tu les rassembles comment ?</t>
+          <t>Le seau tape sa jambe, à chaque pas. Au kiosque, les marches sont trop hautes. Le goûter, là-haut. Le seau tape une marche, trop haute. Un vent passe, tout froid. Trop haut, trop loin. Le canard rond ne monte pas. Le mince commence, puis recule. Ils ne viennent pas. Le kiosque est trop loin de l'eau. Tu les rassembles comment ?</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -15251,9 +15266,10 @@
         <is>
           <t>narrateur|Le seau tape sa jambe, à chaque pas.
 narrateur|Au kiosque, les marches sont trop hautes.
+enfant-m|Le goûter, là-haut.
 narrateur|Le seau tape une marche, trop haute.
-enfant-m|Le goûter, là-haut.
 narrateur|Un vent passe, tout froid.
+maman|Trop haut, trop loin.
 narrateur|Le canard rond ne monte pas.
 narrateur|Le mince commence, puis recule.
 enfant-m|Ils ne viennent pas.
@@ -16518,7 +16534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -16561,6 +16577,13 @@
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>